<commit_message>
Fix Summary tab queries to pull from Light tab
- A15 QUERY: corrected range from Light!A15:K500 to Light!A10:K500
  (data starts at row 10, was skipping first 5 rows)
- B15 FILTER: replaced stale 'Detailed workplan' / 'Detailed Workplan
  Summary' sheet references with Light / Summary

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoldCure Workplan2.xlsx
+++ b/MoldCure Workplan2.xlsx
@@ -29484,7 +29484,7 @@
       <c r="A15" s="38" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("ARRAY_CONSTRAIN(
   QUERY(
-    Light!A15:K500,
+    Light!A10:K500,
     ""select A,B,C,D,E,F,G,H,I
      where G &gt;= "" &amp; Summary!A11 &amp; ""
        and I &lt;= "" &amp; Summary!B11 &amp; ""
@@ -29510,7 +29510,7 @@
       <c r="K15" s="42"/>
       <c r="L15" s="42"/>
       <c r="M15" s="38" t="str">
-        <f t="array" ref="M15">_xlws.FILTER('Detailed workplan'!R:W, ('Detailed workplan'!G:G='Detailed Workplan Summary'!D3)*('Detailed workplan'!J:J='Detailed Workplan Summary'!E3),"NA")</f>
+        <f t="array" ref="M15">_xlws.FILTER(Light!R:W, (Light!G:G=Summary!D3)*(Light!J:J=Summary!E3),"NA")</f>
         <v>#NAME?</v>
       </c>
       <c r="N15" s="39"/>

</xml_diff>

<commit_message>
Replace Google Sheets QUERY/DUMMYFUNCTION with native Excel FILTER+SORT
QUERY is Google Sheets-only and always errors in Excel via DUMMYFUNCTION.
Replaced A15 with IFERROR(SORT(FILTER(...))) using the same filtering
logic: date range, exclude Complete, optional assigned-to and priority.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoldCure Workplan2.xlsx
+++ b/MoldCure Workplan2.xlsx
@@ -29481,22 +29481,8 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="38" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("ARRAY_CONSTRAIN(
-  QUERY(
-    Light!A10:K500,
-    ""select A,B,C,D,E,F,G,H,I
-     where G &gt;= "" &amp; Summary!A11 &amp; ""
-       and I &lt;= "" &amp; Summary!B11 &amp; ""
-       and D &lt;&gt; 'Complete'
-       and ("" &amp; IF(Summary!D11="""",""true"",""C = '"" &amp; Summary!D11 &amp; ""'"&amp;""") &amp; "")
-       and ("" &amp; IF(Summary!E11="""",""true"",""E = '"" &amp; Summary!E11 &amp; ""'"") &amp; "")
-     order by H asc"",
-    0
-  ),
-80, 8)
-"),"#N/A")</f>
-        <v>#N/A</v>
+      <c r="A15" s="38">
+        <f>IFERROR(SORT(FILTER(Light!A10:I500,(Light!G10:G500&gt;=Summary!A11)*(Light!I10:I500&lt;=Summary!B11)*(Light!D10:D500&lt;&gt;"Complete")*IF(Summary!D11="",1,Light!C10:C500=Summary!D11)*IF(Summary!E11="",1,Light!E10:E500=Summary!E11)),8,1),"")</f>
       </c>
       <c r="B15" s="19"/>
       <c r="C15" s="19"/>

</xml_diff>